<commit_message>
fix: use updated Production requirements template font
</commit_message>
<xml_diff>
--- a/src/assets/production-templates/ROMIKU生产单模板.xlsx
+++ b/src/assets/production-templates/ROMIKU生产单模板.xlsx
@@ -78,7 +78,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -119,6 +119,20 @@
       <sz val="16"/>
       <color rgb="FFFF0000"/>
       <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体-简"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -642,28 +656,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -672,123 +677,132 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -826,19 +840,16 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1358,36 +1369,36 @@
       <c r="A6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="16"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" ht="88" customHeight="1" spans="1:7">
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
     </row>
     <row r="8" ht="57" customHeight="1" spans="1:7">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1401,7 +1412,7 @@
   <pageSetup paperSize="9" scale="62" orientation="portrait"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="C6:G6 A7:G9 G5 D5:E5" numberStoredAsText="1"/>
+    <ignoredError sqref="D5:E5 G5 A7:G9 D6:G6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add saved Production barcodes and adopt final XLSX template
</commit_message>
<xml_diff>
--- a/src/assets/production-templates/ROMIKU生产单模板.xlsx
+++ b/src/assets/production-templates/ROMIKU生产单模板.xlsx
@@ -2,13 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <bookViews>
     <workbookView windowHeight="15280"/>
   </bookViews>
   <sheets>
     <sheet name="ROMIKU PI" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROMIKU PI'!$A1:$H6</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>正唛</t>
   </si>
@@ -35,7 +38,7 @@
     <t>侧唛</t>
   </si>
   <si>
-    <t>小标签</t>
+    <t>小标签格式</t>
   </si>
   <si>
     <t>贴标要求</t>
@@ -45,6 +48,9 @@
   </si>
   <si>
     <t>货号</t>
+  </si>
+  <si>
+    <t>条形码</t>
   </si>
   <si>
     <t xml:space="preserve"> 图片</t>
@@ -81,8 +87,10 @@
   <fonts count="30">
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -99,19 +107,25 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Songti SC Regular"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
       <sz val="20"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="20"/>
+      <name val="Carlito"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Songti SC Regular"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <name val="Songti SC Regular"/>
       <charset val="134"/>
     </font>
@@ -126,13 +140,6 @@
       <sz val="18"/>
       <color rgb="FFFF0000"/>
       <name val="宋体-简"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -499,21 +506,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -542,6 +534,21 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -652,10 +659,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="50">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -800,60 +805,59 @@
     <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
     <cellStyle name="货币" xfId="2" builtinId="4"/>
@@ -903,223 +907,8 @@
     <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-  </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
-    </tableStyle>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1276,143 +1065,156 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="31.4230769230769" customWidth="1"/>
-    <col min="3" max="3" width="30.5673076923077" customWidth="1"/>
-    <col min="4" max="4" width="31.8269230769231" customWidth="1"/>
-    <col min="5" max="5" width="12.3173076923077" customWidth="1"/>
-    <col min="6" max="6" width="11.4711538461538" customWidth="1"/>
-    <col min="7" max="7" width="13.75" customWidth="1"/>
+    <col min="2" max="2" width="31.421875" customWidth="1"/>
+    <col min="3" max="4" width="30.5703125" customWidth="1"/>
+    <col min="5" max="5" width="31.828125" customWidth="1"/>
+    <col min="6" max="6" width="12.3203125" customWidth="1"/>
+    <col min="7" max="7" width="11.46875" customWidth="1"/>
+    <col min="8" max="8" width="13.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:7">
-      <c r="B1" s="1" t="s">
+    <row r="1" ht="35" customHeight="1" spans="1:8">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
-    <row r="2" ht="137" customHeight="1" spans="1:7">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+    <row r="2" ht="137" customHeight="1" spans="1:8">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
     </row>
-    <row r="3" ht="34" customHeight="1" spans="1:7">
-      <c r="A3" s="8" t="s">
+    <row r="3" ht="34" customHeight="1" spans="1:8">
+      <c r="A3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="11" t="s">
         <v>10</v>
       </c>
+      <c r="H3" s="11" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="4" ht="112" customHeight="1" spans="1:7">
-      <c r="A4" s="9"/>
+    <row r="4" ht="112" customHeight="1" spans="1:8">
+      <c r="A4" s="9">
+        <v>1</v>
+      </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="9">
-        <f>E4*F4</f>
-        <v>0</v>
-      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
-    <row r="5" ht="35" customHeight="1" spans="1:7">
-      <c r="A5" s="10" t="s">
+    <row r="5" ht="35" customHeight="1" spans="1:8">
+      <c r="A5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="13">
+        <v>1</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11">
-        <f>SUM(E4:E4)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="11"/>
+      <c r="H5" s="13">
+        <v>32</v>
+      </c>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:7">
-      <c r="A6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
+    <row r="6" ht="50" customHeight="1" spans="1:8">
+      <c r="A6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
       <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
-    <row r="7" ht="88" customHeight="1" spans="1:7">
+    <row r="7" ht="88" customHeight="1" spans="1:8">
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
     </row>
-    <row r="8" ht="57" customHeight="1" spans="1:7">
+    <row r="8" ht="57" customHeight="1" spans="1:8">
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="A5:D5"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C6:H6"/>
   </mergeCells>
   <pageMargins left="0.751388888888889" right="0.751388888888889" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="62" orientation="portrait"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
   <headerFooter/>
-  <ignoredErrors>
-    <ignoredError sqref="D5:E5 G5 A7:G9 D6:G6" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>